<commit_message>
working on getting nn species ratios for all sites
</commit_message>
<xml_diff>
--- a/species_list_nov.xlsx
+++ b/species_list_nov.xlsx
@@ -351,7 +351,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:A43"/>
+  <dimension ref="A1:A44"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" s="1" customFormat="1">
@@ -581,75 +581,82 @@
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>EROCIC</t>
+          <t>BRANIG</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>LUP Sp.</t>
+          <t>EROCIC</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>CARPYC</t>
+          <t>LUP Sp.</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>LUP sp.</t>
+          <t>CARPYC</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>ACMAME</t>
+          <t>LUP sp.</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>HEMFAS</t>
+          <t>ACMAME</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>GALAPA</t>
+          <t>HEMFAS</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>LYSARV</t>
+          <t>GALAPA</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>JEPPAR</t>
+          <t>LYSARV</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>MADELE</t>
+          <t>JEPPAR</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
+        <is>
+          <t>MADELE</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="inlineStr">
         <is>
           <t>LESFIL</t>
         </is>

</xml_diff>